<commit_message>
Publish 1009 environment-shared residual revision
Synchronize the 224-record dataset, latest environmental residual rules and all 290 reference artifacts. Split the analysis into twelve source files with minimal comments and retain the original algorithm, candidates and seeds. Correct the prospective launcher argument handling.

The complete public workflow matches the supplied full_20261008_182317_470433 run: 141 tables, 170 checkpoints and 4,838,654 numeric values with zero differences; frozen inference also matches for all 224 conditions.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plot_Data_Verified" sheetId="1" r:id="R10cd4729b895477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plot_Data" sheetId="2" r:id="R9d84c56d341d4496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plot_Data_Original" sheetId="3" r:id="Rccfffdd433c54001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plot_Data_Verified" sheetId="1" r:id="R45272ad5ffa74631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plot_Data" sheetId="2" r:id="R2731a4977ee74aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plot_Data_Original" sheetId="3" r:id="Re666c6a6416a4413"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DataTable1" displayName="DataTable1" ref="A1:AF224" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DataTable1" displayName="DataTable1" ref="A1:AF225" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="32">
     <x:tableColumn id="1" name="row_id"/>
     <x:tableColumn id="2" name="T_C"/>
@@ -213,7 +213,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DataTable2" displayName="DataTable2" ref="A1:H247" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DataTable2" displayName="DataTable2" ref="A1:H248" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="row_id"/>
     <x:tableColumn id="2" name="record_equivalence_id"/>
@@ -229,7 +229,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="DataTable3" displayName="DataTable3" ref="A1:C247" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="DataTable3" displayName="DataTable3" ref="A1:C248" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="row_id"/>
     <x:tableColumn id="2" name="Nf_cycles"/>
@@ -22035,38 +22035,100 @@
       </x:c>
     </x:row>
     <x:row r="225" ht="25" customHeight="1">
-      <x:c r="A225" s="12"/>
-      <x:c r="B225" s="12"/>
-      <x:c r="C225" s="14"/>
-      <x:c r="D225" s="16"/>
-      <x:c r="E225" s="16"/>
-      <x:c r="F225" s="16"/>
-      <x:c r="G225" s="18"/>
-      <x:c r="H225" s="12"/>
-      <x:c r="I225" s="21"/>
-      <x:c r="J225" s="20"/>
-      <x:c r="K225" s="20"/>
-      <x:c r="L225" s="20"/>
-      <x:c r="M225" s="20"/>
-      <x:c r="N225" s="21"/>
+      <x:c r="A225" s="12" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="B225" s="12" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C225" s="14" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D225" s="16" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E225" s="16" t="n">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="F225" s="16" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G225" s="18" t="n">
+        <x:v>0.628</x:v>
+      </x:c>
+      <x:c r="H225" s="12" t="n">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="I225" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J225" s="20" t="str">
+        <x:v>2D_woven</x:v>
+      </x:c>
+      <x:c r="K225" s="20" t="str">
+        <x:v>2D</x:v>
+      </x:c>
+      <x:c r="L225" s="20" t="str">
+        <x:v>air_or_oxygen</x:v>
+      </x:c>
+      <x:c r="M225" s="20" t="str">
+        <x:v>RT/T&lt;=80</x:v>
+      </x:c>
+      <x:c r="N225" s="19" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="O225" s="12"/>
-      <x:c r="P225" s="20"/>
-      <x:c r="Q225" s="20"/>
-      <x:c r="R225" s="12"/>
-      <x:c r="S225" s="12"/>
-      <x:c r="T225" s="20"/>
-      <x:c r="U225" s="12"/>
-      <x:c r="V225" s="12"/>
-      <x:c r="W225" s="20"/>
-      <x:c r="X225" s="20"/>
-      <x:c r="Y225" s="20"/>
-      <x:c r="Z225" s="20"/>
-      <x:c r="AA225" s="20"/>
-      <x:c r="AB225" s="20"/>
-      <x:c r="AC225" s="20"/>
-      <x:c r="AD225" s="20"/>
-      <x:c r="AE225" s="20"/>
-      <x:c r="AF225" s="20"/>
+      <x:c r="P225" s="20" t="str">
+        <x:v>EQ-R315</x:v>
+      </x:c>
+      <x:c r="Q225" s="20" t="str">
+        <x:v>right_censored_likelihood_training</x:v>
+      </x:c>
+      <x:c r="R225" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S225" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T225" s="20" t="str">
+        <x:v>right_censored</x:v>
+      </x:c>
+      <x:c r="U225" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V225" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W225" s="20" t="str">
+        <x:v>primary_experiment</x:v>
+      </x:c>
+      <x:c r="X225" s="20" t="str">
+        <x:v>primary_table_secondary_UTS_reference</x:v>
+      </x:c>
+      <x:c r="Y225" s="20" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="Z225" s="20" t="str">
+        <x:v>no_confirmed_duplicate</x:v>
+      </x:c>
+      <x:c r="AA225" s="20" t="str">
+        <x:v>&gt;1000000</x:v>
+      </x:c>
+      <x:c r="AB225" s="20" t="str">
+        <x:v>CAMPAIGN-MIN-2D-CSIC-RT</x:v>
+      </x:c>
+      <x:c r="AC225" s="20" t="str">
+        <x:v>J. B. Min | 2013 | Micromechanics Fatigue Damage Analysis Modeling for Fabric Reinforced Ceramic Matrix Composites</x:v>
+      </x:c>
+      <x:c r="AD225" s="20" t="str">
+        <x:v>https://ntrs.nasa.gov/citations/20130014831; Li2016 doi:10.1007/s10443-016-9492-5</x:v>
+      </x:c>
+      <x:c r="AE225" s="20" t="str">
+        <x:v>NASA/TM-2013-217870, Table 5 p.17, row 05: 314 MPa, &gt;1,000,000 cycles; 23 C, R=0.1, 5 Hz. Recorded as right-censored at 1,000,000 cycles. UTS 500 MPa follows the same Li2016 normalization reference as the other Min records.</x:v>
+      </x:c>
+      <x:c r="AF225" s="20" t="str">
+        <x:v>Li2016 PDF p10 / journal p922, section4.1.1 explicitly reports500MPa. Retain as Li reported normalization reference, not a newly verified original experimental mean.</x:v>
+      </x:c>
     </x:row>
     <x:row r="226" ht="25" customHeight="1">
       <x:c r="A226" s="12"/>
@@ -22241,7 +22303,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9f9068c38c4489"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21bc02149ab4170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28683,14 +28745,30 @@
       </x:c>
     </x:row>
     <x:row r="248" ht="25" customHeight="1">
-      <x:c r="A248" s="12"/>
-      <x:c r="B248" s="20"/>
-      <x:c r="C248" s="21"/>
-      <x:c r="D248" s="20"/>
-      <x:c r="E248" s="20"/>
-      <x:c r="F248" s="20"/>
-      <x:c r="G248" s="20"/>
-      <x:c r="H248" s="20"/>
+      <x:c r="A248" s="12" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="B248" s="20" t="str">
+        <x:v>EQ-R315</x:v>
+      </x:c>
+      <x:c r="C248" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D248" s="20" t="str">
+        <x:v>primary_experiment</x:v>
+      </x:c>
+      <x:c r="E248" s="20" t="str">
+        <x:v>primary_table_secondary_UTS_reference</x:v>
+      </x:c>
+      <x:c r="F248" s="20" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G248" s="20" t="str">
+        <x:v>no_confirmed_duplicate</x:v>
+      </x:c>
+      <x:c r="H248" s="20" t="str">
+        <x:v>J. B. Min | 2013 | Micromechanics Fatigue Damage Analysis Modeling for Fabric Reinforced Ceramic Matrix Composites</x:v>
+      </x:c>
     </x:row>
     <x:row r="249" ht="25" customHeight="1">
       <x:c r="A249" s="12"/>
@@ -28745,7 +28823,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ea703bc76049ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R339cabcb27b64513"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31477,9 +31555,15 @@
       </x:c>
     </x:row>
     <x:row r="248" ht="25" customHeight="1">
-      <x:c r="A248" s="12"/>
-      <x:c r="B248" s="12"/>
-      <x:c r="C248" s="21"/>
+      <x:c r="A248" s="12" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="B248" s="12" t="n">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="C248" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="249" ht="25" customHeight="1">
       <x:c r="A249" s="12"/>
@@ -31509,7 +31593,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb919099e52fa48a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf19783ff544315"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>